<commit_message>
Add 23 terms to Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O675"/>
+  <dimension ref="A1:O698"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37822,6 +37822,1073 @@
         </is>
       </c>
     </row>
+    <row r="676">
+      <c r="A676" t="inlineStr"/>
+      <c r="B676" t="inlineStr"/>
+      <c r="C676" t="inlineStr"/>
+      <c r="D676" t="inlineStr"/>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>studlab</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Study identifier</t>
+        </is>
+      </c>
+      <c r="G676" t="inlineStr">
+        <is>
+          <t>GMHO:0000211</t>
+        </is>
+      </c>
+      <c r="H676" t="inlineStr">
+        <is>
+          <t>study identification</t>
+        </is>
+      </c>
+      <c r="I676" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A textual entity intended to identify a particular study. </t>
+        </is>
+      </c>
+      <c r="J676" t="inlineStr">
+        <is>
+          <t>textual entity</t>
+        </is>
+      </c>
+      <c r="K676" t="inlineStr">
+        <is>
+          <t>Research methods</t>
+        </is>
+      </c>
+      <c r="L676" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M676" t="inlineStr"/>
+      <c r="N676" t="inlineStr"/>
+      <c r="O676" t="inlineStr"/>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr"/>
+      <c r="B677" t="inlineStr"/>
+      <c r="C677" t="inlineStr"/>
+      <c r="D677" t="inlineStr"/>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>sa_outcome</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Social anxiety scale</t>
+        </is>
+      </c>
+      <c r="G677" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H677" t="inlineStr">
+        <is>
+          <t>social anxiety scale</t>
+        </is>
+      </c>
+      <c r="I677" t="inlineStr">
+        <is>
+          <t>An anxiety scale that is used to measure social anxiety symptom severity.</t>
+        </is>
+      </c>
+      <c r="J677" t="inlineStr">
+        <is>
+          <t>anxiety scale</t>
+        </is>
+      </c>
+      <c r="K677" t="inlineStr">
+        <is>
+          <t>Intervention outcomes and spillover effects</t>
+        </is>
+      </c>
+      <c r="L677" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M677" t="inlineStr"/>
+      <c r="N677" t="inlineStr"/>
+      <c r="O677" t="inlineStr"/>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr"/>
+      <c r="B678" t="inlineStr"/>
+      <c r="C678" t="inlineStr"/>
+      <c r="D678" t="inlineStr"/>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Type of bias training intervention</t>
+        </is>
+      </c>
+      <c r="G678" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H678" t="inlineStr">
+        <is>
+          <t>cognitive bias modification intervention</t>
+        </is>
+      </c>
+      <c r="I678" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An intervention content that uses tasks to assess and modify a person’s cognitive bias dispositions. </t>
+        </is>
+      </c>
+      <c r="J678" t="inlineStr">
+        <is>
+          <t>intervention content</t>
+        </is>
+      </c>
+      <c r="K678" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="L678" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M678" t="inlineStr"/>
+      <c r="N678" t="inlineStr"/>
+      <c r="O678" t="inlineStr"/>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr"/>
+      <c r="B679" t="inlineStr"/>
+      <c r="C679" t="inlineStr"/>
+      <c r="D679" t="inlineStr"/>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>intervention</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Type of bias training intervention</t>
+        </is>
+      </c>
+      <c r="G679" t="inlineStr">
+        <is>
+          <t>GMHO:0000241</t>
+        </is>
+      </c>
+      <c r="H679" t="inlineStr">
+        <is>
+          <t>mental health intervention content</t>
+        </is>
+      </c>
+      <c r="I679" t="inlineStr">
+        <is>
+          <t>An intervention content that is part of a mental health intervention.</t>
+        </is>
+      </c>
+      <c r="J679" t="inlineStr">
+        <is>
+          <t>intervention content</t>
+        </is>
+      </c>
+      <c r="K679" t="inlineStr">
+        <is>
+          <t>Intervention content and delivery</t>
+        </is>
+      </c>
+      <c r="L679" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M679" t="inlineStr"/>
+      <c r="N679" t="inlineStr"/>
+      <c r="O679" t="inlineStr"/>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr"/>
+      <c r="B680" t="inlineStr"/>
+      <c r="C680" t="inlineStr"/>
+      <c r="D680" t="inlineStr"/>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>node</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Study arm</t>
+        </is>
+      </c>
+      <c r="G680" t="inlineStr">
+        <is>
+          <t>GMHO:0000127</t>
+        </is>
+      </c>
+      <c r="H680" t="inlineStr">
+        <is>
+          <t>study arm</t>
+        </is>
+      </c>
+      <c r="I680" t="inlineStr">
+        <is>
+          <t>An information content entity that is about an intervention scenario and designates it as part of an intervention evaluation study.</t>
+        </is>
+      </c>
+      <c r="J680" t="inlineStr">
+        <is>
+          <t>information content entity</t>
+        </is>
+      </c>
+      <c r="K680" t="inlineStr">
+        <is>
+          <t>Research methods</t>
+        </is>
+      </c>
+      <c r="L680" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M680" t="inlineStr"/>
+      <c r="N680" t="inlineStr"/>
+      <c r="O680" t="inlineStr"/>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr"/>
+      <c r="B681" t="inlineStr"/>
+      <c r="C681" t="inlineStr"/>
+      <c r="D681" t="inlineStr"/>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>sa_baseline_n</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Number of participants with baseline evaluation on social anxiety</t>
+        </is>
+      </c>
+      <c r="G681" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H681" t="inlineStr">
+        <is>
+          <t>social anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="I681" t="inlineStr">
+        <is>
+          <t>Anxiety symptom severity that is associated with social anxiety.</t>
+        </is>
+      </c>
+      <c r="J681" t="inlineStr">
+        <is>
+          <t>anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="K681" t="inlineStr">
+        <is>
+          <t>Intervention outcomes and spillover effects</t>
+        </is>
+      </c>
+      <c r="L681" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M681" t="inlineStr"/>
+      <c r="N681" t="inlineStr"/>
+      <c r="O681" t="inlineStr"/>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr"/>
+      <c r="B682" t="inlineStr"/>
+      <c r="C682" t="inlineStr"/>
+      <c r="D682" t="inlineStr"/>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>sa_baseline_n</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Number of participants with baseline evaluation on social anxiety</t>
+        </is>
+      </c>
+      <c r="G682" t="inlineStr">
+        <is>
+          <t>GMHO:0000209</t>
+        </is>
+      </c>
+      <c r="H682" t="inlineStr">
+        <is>
+          <t>measurement datum at baseline</t>
+        </is>
+      </c>
+      <c r="I682" t="inlineStr">
+        <is>
+          <t>Measurement datum that was recorded as baseline data in a study.</t>
+        </is>
+      </c>
+      <c r="J682" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="K682" t="inlineStr">
+        <is>
+          <t>Intervention outcomes and spillover effects</t>
+        </is>
+      </c>
+      <c r="L682" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M682" t="inlineStr"/>
+      <c r="N682" t="inlineStr"/>
+      <c r="O682" t="inlineStr"/>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr"/>
+      <c r="B683" t="inlineStr"/>
+      <c r="C683" t="inlineStr"/>
+      <c r="D683" t="inlineStr"/>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>sa_baseline_n</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Number of participants with baseline evaluation on social anxiety</t>
+        </is>
+      </c>
+      <c r="G683" t="inlineStr">
+        <is>
+          <t>GMHO:0000206</t>
+        </is>
+      </c>
+      <c r="H683" t="inlineStr">
+        <is>
+          <t>number of participants with measurement</t>
+        </is>
+      </c>
+      <c r="I683" t="inlineStr">
+        <is>
+          <t>Number of study participants for whom a measurement was made.</t>
+        </is>
+      </c>
+      <c r="J683" t="inlineStr">
+        <is>
+          <t>number of study participants</t>
+        </is>
+      </c>
+      <c r="K683" t="inlineStr">
+        <is>
+          <t>Intervention outcomes and spillover effects</t>
+        </is>
+      </c>
+      <c r="L683" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M683" t="inlineStr"/>
+      <c r="N683" t="inlineStr"/>
+      <c r="O683" t="inlineStr"/>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr"/>
+      <c r="B684" t="inlineStr"/>
+      <c r="C684" t="inlineStr"/>
+      <c r="D684" t="inlineStr"/>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>sa_endpoint_n</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Number of participants with post-intervention evaluation on social anxiety</t>
+        </is>
+      </c>
+      <c r="G684" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H684" t="inlineStr">
+        <is>
+          <t>social anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="I684" t="inlineStr">
+        <is>
+          <t>Anxiety symptom severity that is associated with social anxiety.</t>
+        </is>
+      </c>
+      <c r="J684" t="inlineStr">
+        <is>
+          <t>anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="K684" t="inlineStr"/>
+      <c r="L684" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M684" t="inlineStr"/>
+      <c r="N684" t="inlineStr"/>
+      <c r="O684" t="inlineStr"/>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr"/>
+      <c r="B685" t="inlineStr"/>
+      <c r="C685" t="inlineStr"/>
+      <c r="D685" t="inlineStr"/>
+      <c r="E685" t="inlineStr">
+        <is>
+          <t>sa_endpoint_n</t>
+        </is>
+      </c>
+      <c r="F685" t="inlineStr">
+        <is>
+          <t>Number of participants with post-intervention evaluation on social anxiety</t>
+        </is>
+      </c>
+      <c r="G685" t="inlineStr">
+        <is>
+          <t>GMHO:0000204</t>
+        </is>
+      </c>
+      <c r="H685" t="inlineStr">
+        <is>
+          <t>measurement datum at post-intervention</t>
+        </is>
+      </c>
+      <c r="I685" t="inlineStr">
+        <is>
+          <t>Measurement datum that was recorded as post-intervention data in a study.</t>
+        </is>
+      </c>
+      <c r="J685" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="K685" t="inlineStr"/>
+      <c r="L685" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M685" t="inlineStr"/>
+      <c r="N685" t="inlineStr"/>
+      <c r="O685" t="inlineStr"/>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr"/>
+      <c r="B686" t="inlineStr"/>
+      <c r="C686" t="inlineStr"/>
+      <c r="D686" t="inlineStr"/>
+      <c r="E686" t="inlineStr">
+        <is>
+          <t>sa_endpoint_n</t>
+        </is>
+      </c>
+      <c r="F686" t="inlineStr">
+        <is>
+          <t>Number of participants with post-intervention evaluation on social anxiety</t>
+        </is>
+      </c>
+      <c r="G686" t="inlineStr">
+        <is>
+          <t>GMHO:0000206</t>
+        </is>
+      </c>
+      <c r="H686" t="inlineStr">
+        <is>
+          <t>number of participants with measurement</t>
+        </is>
+      </c>
+      <c r="I686" t="inlineStr">
+        <is>
+          <t>Number of study participants for whom a measurement was made.</t>
+        </is>
+      </c>
+      <c r="J686" t="inlineStr">
+        <is>
+          <t>number of study participants</t>
+        </is>
+      </c>
+      <c r="K686" t="inlineStr"/>
+      <c r="L686" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M686" t="inlineStr"/>
+      <c r="N686" t="inlineStr"/>
+      <c r="O686" t="inlineStr"/>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr"/>
+      <c r="B687" t="inlineStr"/>
+      <c r="C687" t="inlineStr"/>
+      <c r="D687" t="inlineStr"/>
+      <c r="E687" t="inlineStr">
+        <is>
+          <t>sa_baseline_mean</t>
+        </is>
+      </c>
+      <c r="F687" t="inlineStr">
+        <is>
+          <t>Mean baseline social anxiety</t>
+        </is>
+      </c>
+      <c r="G687" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H687" t="inlineStr">
+        <is>
+          <t>social anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="I687" t="inlineStr">
+        <is>
+          <t>Anxiety symptom severity that is associated with social anxiety.</t>
+        </is>
+      </c>
+      <c r="J687" t="inlineStr">
+        <is>
+          <t>anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="K687" t="inlineStr"/>
+      <c r="L687" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M687" t="inlineStr"/>
+      <c r="N687" t="inlineStr"/>
+      <c r="O687" t="inlineStr"/>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr"/>
+      <c r="B688" t="inlineStr"/>
+      <c r="C688" t="inlineStr"/>
+      <c r="D688" t="inlineStr"/>
+      <c r="E688" t="inlineStr">
+        <is>
+          <t>sa_baseline_mean</t>
+        </is>
+      </c>
+      <c r="F688" t="inlineStr">
+        <is>
+          <t>Mean baseline social anxiety</t>
+        </is>
+      </c>
+      <c r="G688" t="inlineStr">
+        <is>
+          <t>GMHO:0000209</t>
+        </is>
+      </c>
+      <c r="H688" t="inlineStr">
+        <is>
+          <t>measurement datum at baseline</t>
+        </is>
+      </c>
+      <c r="I688" t="inlineStr">
+        <is>
+          <t>Measurement datum that was recorded as baseline data in a study.</t>
+        </is>
+      </c>
+      <c r="J688" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="K688" t="inlineStr"/>
+      <c r="L688" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M688" t="inlineStr"/>
+      <c r="N688" t="inlineStr"/>
+      <c r="O688" t="inlineStr"/>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr"/>
+      <c r="B689" t="inlineStr"/>
+      <c r="C689" t="inlineStr"/>
+      <c r="D689" t="inlineStr"/>
+      <c r="E689" t="inlineStr">
+        <is>
+          <t>sa_baseline_mean</t>
+        </is>
+      </c>
+      <c r="F689" t="inlineStr">
+        <is>
+          <t>Mean baseline social anxiety</t>
+        </is>
+      </c>
+      <c r="G689" t="inlineStr">
+        <is>
+          <t>OBI:0000679</t>
+        </is>
+      </c>
+      <c r="H689" t="inlineStr">
+        <is>
+          <t>average value</t>
+        </is>
+      </c>
+      <c r="I689" t="inlineStr">
+        <is>
+          <t>A data item that is produced as the output of an averaging data transformation and represents the average value of the input data.</t>
+        </is>
+      </c>
+      <c r="J689" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="K689" t="inlineStr"/>
+      <c r="L689" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M689" t="inlineStr"/>
+      <c r="N689" t="inlineStr"/>
+      <c r="O689" t="inlineStr"/>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr"/>
+      <c r="B690" t="inlineStr"/>
+      <c r="C690" t="inlineStr"/>
+      <c r="D690" t="inlineStr"/>
+      <c r="E690" t="inlineStr">
+        <is>
+          <t>sa_endpoint_mean</t>
+        </is>
+      </c>
+      <c r="F690" t="inlineStr">
+        <is>
+          <t>Mean post-intervention social anxiety</t>
+        </is>
+      </c>
+      <c r="G690" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H690" t="inlineStr">
+        <is>
+          <t>social anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="I690" t="inlineStr">
+        <is>
+          <t>Anxiety symptom severity that is associated with social anxiety.</t>
+        </is>
+      </c>
+      <c r="J690" t="inlineStr">
+        <is>
+          <t>anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="K690" t="inlineStr"/>
+      <c r="L690" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M690" t="inlineStr"/>
+      <c r="N690" t="inlineStr"/>
+      <c r="O690" t="inlineStr"/>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr"/>
+      <c r="B691" t="inlineStr"/>
+      <c r="C691" t="inlineStr"/>
+      <c r="D691" t="inlineStr"/>
+      <c r="E691" t="inlineStr">
+        <is>
+          <t>sa_endpoint_mean</t>
+        </is>
+      </c>
+      <c r="F691" t="inlineStr">
+        <is>
+          <t>Mean post-intervention social anxiety</t>
+        </is>
+      </c>
+      <c r="G691" t="inlineStr">
+        <is>
+          <t>GMHO:0000204</t>
+        </is>
+      </c>
+      <c r="H691" t="inlineStr">
+        <is>
+          <t>measurement datum at post-intervention</t>
+        </is>
+      </c>
+      <c r="I691" t="inlineStr">
+        <is>
+          <t>Measurement datum that was recorded as post-intervention data in a study.</t>
+        </is>
+      </c>
+      <c r="J691" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="K691" t="inlineStr"/>
+      <c r="L691" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M691" t="inlineStr"/>
+      <c r="N691" t="inlineStr"/>
+      <c r="O691" t="inlineStr"/>
+    </row>
+    <row r="692">
+      <c r="A692" t="inlineStr"/>
+      <c r="B692" t="inlineStr"/>
+      <c r="C692" t="inlineStr"/>
+      <c r="D692" t="inlineStr"/>
+      <c r="E692" t="inlineStr">
+        <is>
+          <t>sa_endpoint_mean</t>
+        </is>
+      </c>
+      <c r="F692" t="inlineStr">
+        <is>
+          <t>Mean post-intervention social anxiety</t>
+        </is>
+      </c>
+      <c r="G692" t="inlineStr">
+        <is>
+          <t>OBI:0000679</t>
+        </is>
+      </c>
+      <c r="H692" t="inlineStr">
+        <is>
+          <t>average value</t>
+        </is>
+      </c>
+      <c r="I692" t="inlineStr">
+        <is>
+          <t>A data item that is produced as the output of an averaging data transformation and represents the average value of the input data.</t>
+        </is>
+      </c>
+      <c r="J692" t="inlineStr">
+        <is>
+          <t>data item</t>
+        </is>
+      </c>
+      <c r="K692" t="inlineStr"/>
+      <c r="L692" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M692" t="inlineStr"/>
+      <c r="N692" t="inlineStr"/>
+      <c r="O692" t="inlineStr"/>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr"/>
+      <c r="B693" t="inlineStr"/>
+      <c r="C693" t="inlineStr"/>
+      <c r="D693" t="inlineStr"/>
+      <c r="E693" t="inlineStr">
+        <is>
+          <t>sa_baseline_sd</t>
+        </is>
+      </c>
+      <c r="F693" t="inlineStr">
+        <is>
+          <t>Standard deviation of baseline social anxiety</t>
+        </is>
+      </c>
+      <c r="G693" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H693" t="inlineStr">
+        <is>
+          <t>social anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="I693" t="inlineStr">
+        <is>
+          <t>Anxiety symptom severity that is associated with social anxiety.</t>
+        </is>
+      </c>
+      <c r="J693" t="inlineStr">
+        <is>
+          <t>anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="K693" t="inlineStr"/>
+      <c r="L693" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M693" t="inlineStr"/>
+      <c r="N693" t="inlineStr"/>
+      <c r="O693" t="inlineStr"/>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr"/>
+      <c r="B694" t="inlineStr"/>
+      <c r="C694" t="inlineStr"/>
+      <c r="D694" t="inlineStr"/>
+      <c r="E694" t="inlineStr">
+        <is>
+          <t>sa_baseline_sd</t>
+        </is>
+      </c>
+      <c r="F694" t="inlineStr">
+        <is>
+          <t>Standard deviation of baseline social anxiety</t>
+        </is>
+      </c>
+      <c r="G694" t="inlineStr">
+        <is>
+          <t>GMHO:0000209</t>
+        </is>
+      </c>
+      <c r="H694" t="inlineStr">
+        <is>
+          <t>measurement datum at baseline</t>
+        </is>
+      </c>
+      <c r="I694" t="inlineStr">
+        <is>
+          <t>Measurement datum that was recorded as baseline data in a study.</t>
+        </is>
+      </c>
+      <c r="J694" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="K694" t="inlineStr"/>
+      <c r="L694" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M694" t="inlineStr"/>
+      <c r="N694" t="inlineStr"/>
+      <c r="O694" t="inlineStr"/>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr"/>
+      <c r="B695" t="inlineStr"/>
+      <c r="C695" t="inlineStr"/>
+      <c r="D695" t="inlineStr"/>
+      <c r="E695" t="inlineStr">
+        <is>
+          <t>sa_baseline_sd</t>
+        </is>
+      </c>
+      <c r="F695" t="inlineStr">
+        <is>
+          <t>Standard deviation of baseline social anxiety</t>
+        </is>
+      </c>
+      <c r="G695" t="inlineStr">
+        <is>
+          <t>OBCS:0000077</t>
+        </is>
+      </c>
+      <c r="H695" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="I695" t="inlineStr">
+        <is>
+          <t>A quantitative confidence value that measures the variability of data around the mean.</t>
+        </is>
+      </c>
+      <c r="J695" t="inlineStr">
+        <is>
+          <t>quantitative confidence value</t>
+        </is>
+      </c>
+      <c r="K695" t="inlineStr"/>
+      <c r="L695" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M695" t="inlineStr"/>
+      <c r="N695" t="inlineStr"/>
+      <c r="O695" t="inlineStr"/>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr"/>
+      <c r="B696" t="inlineStr"/>
+      <c r="C696" t="inlineStr"/>
+      <c r="D696" t="inlineStr"/>
+      <c r="E696" t="inlineStr">
+        <is>
+          <t>sa_endpoint_sd</t>
+        </is>
+      </c>
+      <c r="F696" t="inlineStr">
+        <is>
+          <t>Standard deviation of post-intervention social anxiety</t>
+        </is>
+      </c>
+      <c r="G696" t="inlineStr">
+        <is>
+          <t>NEW</t>
+        </is>
+      </c>
+      <c r="H696" t="inlineStr">
+        <is>
+          <t>social anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="I696" t="inlineStr">
+        <is>
+          <t>Anxiety symptom severity that is associated with social anxiety.</t>
+        </is>
+      </c>
+      <c r="J696" t="inlineStr">
+        <is>
+          <t>anxiety symptom severity</t>
+        </is>
+      </c>
+      <c r="K696" t="inlineStr"/>
+      <c r="L696" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M696" t="inlineStr"/>
+      <c r="N696" t="inlineStr"/>
+      <c r="O696" t="inlineStr"/>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr"/>
+      <c r="B697" t="inlineStr"/>
+      <c r="C697" t="inlineStr"/>
+      <c r="D697" t="inlineStr"/>
+      <c r="E697" t="inlineStr">
+        <is>
+          <t>sa_endpoint_sd</t>
+        </is>
+      </c>
+      <c r="F697" t="inlineStr">
+        <is>
+          <t>Standard deviation of post-intervention social anxiety</t>
+        </is>
+      </c>
+      <c r="G697" t="inlineStr">
+        <is>
+          <t>GMHO:0000204</t>
+        </is>
+      </c>
+      <c r="H697" t="inlineStr">
+        <is>
+          <t>measurement datum at post-intervention</t>
+        </is>
+      </c>
+      <c r="I697" t="inlineStr">
+        <is>
+          <t>Measurement datum that was recorded as post-intervention data in a study.</t>
+        </is>
+      </c>
+      <c r="J697" t="inlineStr">
+        <is>
+          <t>measurement datum</t>
+        </is>
+      </c>
+      <c r="K697" t="inlineStr"/>
+      <c r="L697" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M697" t="inlineStr"/>
+      <c r="N697" t="inlineStr"/>
+      <c r="O697" t="inlineStr"/>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr"/>
+      <c r="B698" t="inlineStr"/>
+      <c r="C698" t="inlineStr"/>
+      <c r="D698" t="inlineStr"/>
+      <c r="E698" t="inlineStr">
+        <is>
+          <t>sa_endpoint_sd</t>
+        </is>
+      </c>
+      <c r="F698" t="inlineStr">
+        <is>
+          <t>Standard deviation of post-intervention social anxiety</t>
+        </is>
+      </c>
+      <c r="G698" t="inlineStr">
+        <is>
+          <t>OBCS:0000077</t>
+        </is>
+      </c>
+      <c r="H698" t="inlineStr">
+        <is>
+          <t>standard deviation</t>
+        </is>
+      </c>
+      <c r="I698" t="inlineStr">
+        <is>
+          <t>A quantitative confidence value that measures the variability of data around the mean.</t>
+        </is>
+      </c>
+      <c r="J698" t="inlineStr">
+        <is>
+          <t>quantitative confidence value</t>
+        </is>
+      </c>
+      <c r="K698" t="inlineStr"/>
+      <c r="L698" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="M698" t="inlineStr"/>
+      <c r="N698" t="inlineStr"/>
+      <c r="O698" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update 11 terms in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -17093,7 +17093,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Mean post-intervention weight</t>
+          <t>Mean change in post-intervention weight</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -17160,7 +17160,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Mean post-intervention weight</t>
+          <t>Mean change in post-intervention weight</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -17227,7 +17227,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Mean post-intervention weight</t>
+          <t>Mean change in post-intervention weight</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -17686,7 +17686,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Scale for prolactin</t>
+          <t>Unit of prolactin</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -17753,22 +17753,22 @@
       </c>
       <c r="G262" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J262" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K262" t="inlineStr">
@@ -17954,22 +17954,22 @@
       </c>
       <c r="G265" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H265" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I265" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J265" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K265" t="inlineStr">
@@ -18155,22 +18155,22 @@
       </c>
       <c r="G268" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H268" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I268" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J268" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K268" t="inlineStr">
@@ -18356,22 +18356,22 @@
       </c>
       <c r="G271" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H271" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I271" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J271" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K271" t="inlineStr">
@@ -18619,22 +18619,22 @@
       </c>
       <c r="G275" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H275" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -31712,22 +31712,22 @@
       </c>
       <c r="G514" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H514" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I514" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J514" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K514" t="inlineStr">
@@ -35240,27 +35240,27 @@
       </c>
       <c r="F578" t="inlineStr">
         <is>
-          <t>Scale for prolactin</t>
+          <t>Unit of prolactin</t>
         </is>
       </c>
       <c r="G578" t="inlineStr">
         <is>
-          <t>OBA:1000952</t>
+          <t>CMO:0001822</t>
         </is>
       </c>
       <c r="H578" t="inlineStr">
         <is>
-          <t>prolactin level</t>
+          <t>blood prolactin level</t>
         </is>
       </c>
       <c r="I578" t="inlineStr">
         <is>
-          <t>The amount of a prolactin.</t>
+          <t>The amount of prolactin found in a specified volume of blood, the fluid that circulates through the heart, arteries, capillaries and veins carrying nutrients and oxygen to the body tissues and metabolites away from them. Prolactin is a peptide hormone which is secreted by the anterior pituitary and is involved in lactation, growth regulation for tissues including cells of the immune system, and possibly supression of apoptosis. A peptide hormone is a complex organic compound that contains carbon, hydrogen, oxygen, nitrogen, and sulfur consisting of alpha-amino acids joined by peptide linkages, and that is produced in one part or organ of the body and initiates or regulates the activity of an organ or a group of cells in another part of the body.</t>
         </is>
       </c>
       <c r="J578" t="inlineStr">
         <is>
-          <t>protein amount</t>
+          <t>blood peptide hormone level</t>
         </is>
       </c>
       <c r="K578" t="inlineStr">

</xml_diff>

<commit_message>
Update 5 terms in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -17093,7 +17093,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Mean change in post-intervention weight</t>
+          <t>Mean post-intervention weight</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -17160,7 +17160,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Mean change in post-intervention weight</t>
+          <t>Mean post-intervention weight</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -17227,7 +17227,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Mean change in post-intervention weight</t>
+          <t>Mean post-intervention weight</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -17686,7 +17686,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Unit of prolactin</t>
+          <t>Scale for prolactin</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -35240,7 +35240,7 @@
       </c>
       <c r="F578" t="inlineStr">
         <is>
-          <t>Unit of prolactin</t>
+          <t>Scale for prolactin</t>
         </is>
       </c>
       <c r="G578" t="inlineStr">

</xml_diff>

<commit_message>
Update 4 terms in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -17093,7 +17093,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Mean post-intervention weight</t>
+          <t>Mean change in post-intervention weight</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -17160,7 +17160,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Mean post-intervention weight</t>
+          <t>Mean change in post-intervention weight</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -17227,7 +17227,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Mean post-intervention weight</t>
+          <t>Mean change in post-intervention weight</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -17686,7 +17686,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Scale for prolactin</t>
+          <t>Unit of prolactin</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">

</xml_diff>

<commit_message>
Update 6 terms in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -38721,7 +38721,7 @@
       </c>
       <c r="F699" t="inlineStr">
         <is>
-          <t>Depression scale</t>
+          <t>Scale for depression</t>
         </is>
       </c>
       <c r="G699" t="inlineStr">
@@ -38980,7 +38980,7 @@
       </c>
       <c r="F706" t="inlineStr">
         <is>
-          <t>Mean baseline social depression</t>
+          <t>Mean baseline depression</t>
         </is>
       </c>
       <c r="G706" t="inlineStr">
@@ -39017,7 +39017,7 @@
       </c>
       <c r="F707" t="inlineStr">
         <is>
-          <t>Mean baseline social depression</t>
+          <t>Mean baseline depression</t>
         </is>
       </c>
       <c r="G707" t="inlineStr">
@@ -39054,7 +39054,7 @@
       </c>
       <c r="F708" t="inlineStr">
         <is>
-          <t>Mean baseline social depression</t>
+          <t>Mean baseline depression</t>
         </is>
       </c>
       <c r="G708" t="inlineStr">
@@ -41533,7 +41533,7 @@
       </c>
       <c r="F775" t="inlineStr">
         <is>
-          <t>Number of participants for whom dropout was assessed</t>
+          <t>Number of participants for whom drop out was assessed</t>
         </is>
       </c>
       <c r="G775" t="inlineStr">
@@ -41607,7 +41607,7 @@
       </c>
       <c r="F777" t="inlineStr">
         <is>
-          <t>Country of implementation</t>
+          <t>Country of intervention</t>
         </is>
       </c>
       <c r="G777" t="inlineStr">

</xml_diff>

<commit_message>
Update 10 terms in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -38874,7 +38874,7 @@
       </c>
       <c r="G703" t="inlineStr">
         <is>
-          <t>GMHO:0000063</t>
+          <t>GMHO:0000062</t>
         </is>
       </c>
       <c r="H703" t="inlineStr">
@@ -38985,7 +38985,7 @@
       </c>
       <c r="G706" t="inlineStr">
         <is>
-          <t>GMHO:0000064</t>
+          <t>GMHO:0000062</t>
         </is>
       </c>
       <c r="H706" t="inlineStr">
@@ -39096,7 +39096,7 @@
       </c>
       <c r="G709" t="inlineStr">
         <is>
-          <t>GMHO:0000065</t>
+          <t>GMHO:0000062</t>
         </is>
       </c>
       <c r="H709" t="inlineStr">
@@ -39207,7 +39207,7 @@
       </c>
       <c r="G712" t="inlineStr">
         <is>
-          <t>GMHO:0000066</t>
+          <t>GMHO:0000062</t>
         </is>
       </c>
       <c r="H712" t="inlineStr">
@@ -39318,7 +39318,7 @@
       </c>
       <c r="G715" t="inlineStr">
         <is>
-          <t>GMHO:0000067</t>
+          <t>GMHO:0000062</t>
         </is>
       </c>
       <c r="H715" t="inlineStr">
@@ -39577,7 +39577,7 @@
       </c>
       <c r="G722" t="inlineStr">
         <is>
-          <t>GMHO:0000144</t>
+          <t>GMHO:0000143</t>
         </is>
       </c>
       <c r="H722" t="inlineStr">
@@ -39688,7 +39688,7 @@
       </c>
       <c r="G725" t="inlineStr">
         <is>
-          <t>GMHO:0000145</t>
+          <t>GMHO:0000143</t>
         </is>
       </c>
       <c r="H725" t="inlineStr">
@@ -39799,7 +39799,7 @@
       </c>
       <c r="G728" t="inlineStr">
         <is>
-          <t>GMHO:0000146</t>
+          <t>GMHO:0000143</t>
         </is>
       </c>
       <c r="H728" t="inlineStr">
@@ -39910,7 +39910,7 @@
       </c>
       <c r="G731" t="inlineStr">
         <is>
-          <t>GMHO:0000147</t>
+          <t>GMHO:0000143</t>
         </is>
       </c>
       <c r="H731" t="inlineStr">
@@ -40021,7 +40021,7 @@
       </c>
       <c r="G734" t="inlineStr">
         <is>
-          <t>GMHO:0000148</t>
+          <t>GMHO:0000143</t>
         </is>
       </c>
       <c r="H734" t="inlineStr">

</xml_diff>

<commit_message>
Update Row 693 in Mental Health Ontology mapping to LSRs.xlsx
</commit_message>
<xml_diff>
--- a/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
+++ b/Mapping to LSRs/Mental Health Ontology mapping to LSRs.xlsx
@@ -39614,17 +39614,17 @@
       </c>
       <c r="G695" t="inlineStr">
         <is>
-          <t>GMHO:0000274</t>
+          <t>BCIO:008515</t>
         </is>
       </c>
       <c r="H695" t="inlineStr">
         <is>
-          <t>number of mental health intervention contact events</t>
+          <t>number of intervention contact events</t>
         </is>
       </c>
       <c r="I695" t="inlineStr">
         <is>
-          <t>A &lt;data item&gt; that is the number of contact events in a mental health intervention temporal part.</t>
+          <t>A &lt;data item&gt; that is the number of contact events in an intervention temporal part.</t>
         </is>
       </c>
       <c r="J695" t="inlineStr">

</xml_diff>